<commit_message>
Publish monitoring guide and align legacy server contract
</commit_message>
<xml_diff>
--- a/deliverables/GIZMo_Kria_DCS_Intake.xlsx
+++ b/deliverables/GIZMo_Kria_DCS_Intake.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="27120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tag List" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag List" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tag List'!$A$1:$AA$86</definedName>
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="B1:C41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -686,7 +686,7 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>Draft 0.7 requirements intake for joint GIZMo / Slow Controls review</t>
+          <t>Draft 0.8 requirements intake for joint GIZMo / Slow Controls review</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Kria values use the retained 2026-07-27..2026-08-03 permanent SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from the connected ZedBoard on 2026-08-12 plus 27 contiguous deployed-adapter cycles on 2026-08-13; target communication was lost before the 100-cycle acceptance run completed. These sources refine nominal/desired fields but do not replace approved alarm or metrology limits.</t>
+          <t>Kria values use the retained 2026-07-27..2026-08-03 permanent SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from the connected ZedBoard on 2026-08-12 plus 27 contiguous validation-adapter cycles on 2026-08-13; target communication was lost before the 100-cycle acceptance run completed. These sources refine nominal/desired fields but do not replace approved alarm or metrology limits.</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Installed GIZMo runtime or adapter version.</t>
+          <t>Installed GIZMo runtime or OPC UA producer version.</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Boot identifier; changes after target or adapter restart as defined by the platform.</t>
+          <t>Boot identifier; changes after target or OPC UA producer restart as defined by the platform.</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of owned services or adapter processes.</t>
+          <t>Aggregate quality of owned services or OPC UA producer processes.</t>
         </is>
       </c>
       <c r="D84" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Document authenticated legacy threshold control
</commit_message>
<xml_diff>
--- a/deliverables/GIZMo_Kria_DCS_Intake.xlsx
+++ b/deliverables/GIZMo_Kria_DCS_Intake.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="27120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag List" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tag List" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tag List'!$A$1:$AA$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tag List'!$A$1:$AA$88</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Tag List'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Tag List'!$A$1:$AA$86</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Tag List'!$A$1:$AA$88</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C41"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -614,7 +614,7 @@
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
-          <t>opc.tcp://&lt;assigned-host&gt;:4840 (final host/IP assigned by Slow Controls)</t>
+          <t>opc.tcp://&lt;assigned-host&gt;:4840 (final production host/IP assigned by Slow Controls)</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>Draft 0.8 requirements intake for joint GIZMo / Slow Controls review</t>
+          <t>Draft 0.9 requirements intake for joint GIZMo / Slow Controls review</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Kria values use the retained 2026-07-27..2026-08-03 permanent SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from the connected ZedBoard on 2026-08-12 plus 27 contiguous validation-adapter cycles on 2026-08-13; target communication was lost before the 100-cycle acceptance run completed. These sources refine nominal/desired fields but do not replace approved alarm or metrology limits.</t>
+          <t>Kria values use the retained 2026-07-27..2026-08-03 permanent SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from 2026-08-12, 27 contiguous adapter-pilot cycles, and the 2026-08-13 native-server authenticated 100-Ohm idempotent write/readback. The full 100-cycle physical-display acceptance remains open. These sources refine nominal/desired fields but do not replace approved alarm or metrology limits.</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Installed GIZMo runtime or OPC UA producer version.</t>
+          <t>Installed GIZMo runtime or adapter version.</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Boot identifier; changes after target or OPC UA producer restart as defined by the platform.</t>
+          <t>Boot identifier; changes after target or adapter restart as defined by the platform.</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
@@ -6095,7 +6095,11 @@
       <c r="Z63" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="AA63" s="13" t="inlineStr"/>
+      <c r="AA63" s="13" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED. The Kria systemd-timesyncd client queries the directly connected Fermilab-synchronized controls workstation. Manual SetSystemTime is a maintenance fallback, not normal operation.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="42" customHeight="1">
       <c r="A64" s="14" t="inlineStr">
@@ -6105,27 +6109,27 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>UptimeSeconds</t>
+          <t>NtpServiceActive</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>Linux uptime.</t>
+          <t>True when the platform network-time client is running.</t>
         </is>
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.UptimeSeconds</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.NtpServiceActive</t>
         </is>
       </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G64" s="14" t="inlineStr">
@@ -6162,43 +6166,49 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y64" s="14" t="n">
-        <v>10000</v>
+      <c r="Y64" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
       </c>
       <c r="Z64" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="AA64" s="13" t="inlineStr"/>
+      <c r="AA64" s="13" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED. Use with NtpSynchronized and Time.Quality; an active client does not by itself prove valid time.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="42" customHeight="1">
       <c r="A65" s="15" t="inlineStr">
         <is>
-          <t>OperatingSystem</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>CpuUtilizationPercent</t>
+          <t>NtpService</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>CPU utilization between samples.</t>
+          <t>Bounded identification of the configured time synchronization service/source.</t>
         </is>
       </c>
       <c r="D65" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.CpuUtilizationPercent</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.NtpService</t>
         </is>
       </c>
       <c r="E65" s="15" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
@@ -6211,21 +6221,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I65" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="K65" s="15" t="n">
-        <v>35.7</v>
-      </c>
-      <c r="L65" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="M65" s="15" t="n">
-        <v>45</v>
-      </c>
+      <c r="I65" s="15" t="n"/>
+      <c r="J65" s="15" t="n"/>
+      <c r="K65" s="15" t="n"/>
+      <c r="L65" s="15" t="n"/>
+      <c r="M65" s="15" t="n"/>
       <c r="N65" s="15" t="n"/>
       <c r="O65" s="15" t="n"/>
       <c r="P65" s="15" t="n"/>
@@ -6245,47 +6245,49 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y65" s="15" t="n">
-        <v>10000</v>
+      <c r="Y65" s="15" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
       </c>
       <c r="Z65" s="15" t="n">
         <v>10000</v>
       </c>
       <c r="AA65" s="15" t="inlineStr">
         <is>
-          <t>Provisional steady-state commissioning envelope from the retained Kria historian: median 35.68%, 1st--99th percentile minute means 34.30--36.66%; short startup/intervention excursions reached 85.47%. Trend only; no utilization alarm is requested.</t>
+          <t>IMPLEMENTED diagnostic readback. No credentials or unrestricted daemon output are exposed.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="42" customHeight="1">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>OperatingSystem</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>MemoryAvailableBytes</t>
+          <t>UptimeSeconds</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>Physical memory available without swapping.</t>
+          <t>Linux uptime.</t>
         </is>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.MemoryAvailableBytes</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.UptimeSeconds</t>
         </is>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
-          <t>byte</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G66" s="14" t="inlineStr">
@@ -6298,19 +6300,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I66" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="I66" s="14" t="n"/>
       <c r="J66" s="14" t="n"/>
-      <c r="K66" s="14" t="n">
-        <v>3170000000</v>
-      </c>
-      <c r="L66" s="14" t="n">
-        <v>2500000000</v>
-      </c>
-      <c r="M66" s="14" t="n">
-        <v>3400000000</v>
-      </c>
+      <c r="K66" s="14" t="n"/>
+      <c r="L66" s="14" t="n"/>
+      <c r="M66" s="14" t="n"/>
       <c r="N66" s="14" t="n"/>
       <c r="O66" s="14" t="n"/>
       <c r="P66" s="14" t="n"/>
@@ -6334,43 +6328,39 @@
         <v>10000</v>
       </c>
       <c r="Z66" s="14" t="n">
-        <v>10000</v>
-      </c>
-      <c r="AA66" s="13" t="inlineStr">
-        <is>
-          <t>OPC UA built-in type UInt64. Provisional commissioning envelope from the retained Kria historian: median 3.171e9 bytes; absolute observed 2.522e9--3.362e9 bytes. Trend only; no memory alarm is requested.</t>
-        </is>
-      </c>
+        <v>1000</v>
+      </c>
+      <c r="AA66" s="13" t="inlineStr"/>
     </row>
     <row r="67" ht="42" customHeight="1">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>OperatingSystem</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>RuntimeVersion</t>
+          <t>CpuUtilizationPercent</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
         <is>
-          <t>Installed gizmo-runtime package version.</t>
+          <t>CPU utilization between samples.</t>
         </is>
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.RuntimeVersion</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.CpuUtilizationPercent</t>
         </is>
       </c>
       <c r="E67" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="F67" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>%</t>
         </is>
       </c>
       <c r="G67" s="14" t="inlineStr">
@@ -6383,11 +6373,21 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I67" s="14" t="n"/>
-      <c r="J67" s="14" t="n"/>
-      <c r="K67" s="14" t="n"/>
-      <c r="L67" s="14" t="n"/>
-      <c r="M67" s="14" t="n"/>
+      <c r="I67" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="K67" s="14" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="L67" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="M67" s="14" t="n">
+        <v>45</v>
+      </c>
       <c r="N67" s="14" t="n"/>
       <c r="O67" s="14" t="n"/>
       <c r="P67" s="14" t="n"/>
@@ -6407,45 +6407,47 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y67" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
+      <c r="Y67" s="14" t="n">
+        <v>10000</v>
       </c>
       <c r="Z67" s="14" t="n">
-        <v>30000</v>
-      </c>
-      <c r="AA67" s="13" t="inlineStr"/>
+        <v>10000</v>
+      </c>
+      <c r="AA67" s="13" t="inlineStr">
+        <is>
+          <t>Provisional steady-state commissioning envelope from the retained Kria historian: median 35.68%, 1st--99th percentile minute means 34.30--36.66%; short startup/intervention excursions reached 85.47%. Trend only; no utilization alarm is requested.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="42" customHeight="1">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>OperatingSystem</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>OverlayState</t>
+          <t>MemoryAvailableBytes</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
         <is>
-          <t>FPGA overlay state: Running, Degraded, Missing, or unconfirmed.</t>
+          <t>Physical memory available without swapping.</t>
         </is>
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayState</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.MemoryAvailableBytes</t>
         </is>
       </c>
       <c r="E68" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>byte</t>
         </is>
       </c>
       <c r="G68" s="14" t="inlineStr">
@@ -6458,11 +6460,19 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I68" s="14" t="n"/>
+      <c r="I68" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="J68" s="14" t="n"/>
-      <c r="K68" s="14" t="n"/>
-      <c r="L68" s="14" t="n"/>
-      <c r="M68" s="14" t="n"/>
+      <c r="K68" s="14" t="n">
+        <v>3170000000</v>
+      </c>
+      <c r="L68" s="14" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="M68" s="14" t="n">
+        <v>3400000000</v>
+      </c>
       <c r="N68" s="14" t="n"/>
       <c r="O68" s="14" t="n"/>
       <c r="P68" s="14" t="n"/>
@@ -6482,15 +6492,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y68" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
+      <c r="Y68" s="14" t="n">
+        <v>10000</v>
       </c>
       <c r="Z68" s="14" t="n">
-        <v>30000</v>
-      </c>
-      <c r="AA68" s="13" t="inlineStr"/>
+        <v>10000</v>
+      </c>
+      <c r="AA68" s="13" t="inlineStr">
+        <is>
+          <t>OPC UA built-in type UInt64. Provisional commissioning envelope from the retained Kria historian: median 3.171e9 bytes; absolute observed 2.522e9--3.362e9 bytes. Trend only; no memory alarm is requested.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="42" customHeight="1">
       <c r="A69" s="15" t="inlineStr">
@@ -6500,17 +6512,17 @@
       </c>
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>OverlayBitstreamSha256</t>
+          <t>RuntimeVersion</t>
         </is>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>SHA-256 digest of the installed FPGA bitstream.</t>
+          <t>Installed gizmo-runtime package version.</t>
         </is>
       </c>
       <c r="D69" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayBitstreamSha256</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.RuntimeVersion</t>
         </is>
       </c>
       <c r="E69" s="15" t="inlineStr">
@@ -6554,10 +6566,14 @@
       </c>
       <c r="X69" s="15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Y69" s="15" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y69" s="15" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
+      </c>
       <c r="Z69" s="15" t="n">
         <v>30000</v>
       </c>
@@ -6566,22 +6582,22 @@
     <row r="70" ht="42" customHeight="1">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>Calibration</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>OverlayState</t>
         </is>
       </c>
       <c r="C70" s="14" t="inlineStr">
         <is>
-          <t>Validity state of the installed production calibration tables.</t>
+          <t>FPGA overlay state: Running, Degraded, Missing, or unconfirmed.</t>
         </is>
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.State</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayState</t>
         </is>
       </c>
       <c r="E70" s="14" t="inlineStr">
@@ -6641,32 +6657,32 @@
     <row r="71" ht="42" customHeight="1">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>Calibration</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>ConfiguredThresholdOhm</t>
+          <t>OverlayBitstreamSha256</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
-          <t>Threshold persisted in package-owned state.</t>
+          <t>SHA-256 digest of the installed FPGA bitstream.</t>
         </is>
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.ConfiguredThresholdOhm</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayBitstreamSha256</t>
         </is>
       </c>
       <c r="E71" s="14" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F71" s="14" t="inlineStr">
         <is>
-          <t>Ohm</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G71" s="14" t="inlineStr">
@@ -6679,21 +6695,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I71" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" s="14" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="K71" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="L71" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="M71" s="14" t="n">
-        <v>100</v>
-      </c>
+      <c r="I71" s="14" t="n"/>
+      <c r="J71" s="14" t="n"/>
+      <c r="K71" s="14" t="n"/>
+      <c r="L71" s="14" t="n"/>
+      <c r="M71" s="14" t="n"/>
       <c r="N71" s="14" t="n"/>
       <c r="O71" s="14" t="n"/>
       <c r="P71" s="14" t="n"/>
@@ -6710,22 +6716,14 @@
       </c>
       <c r="X71" s="14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Y71" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y71" s="14" t="n"/>
       <c r="Z71" s="14" t="n">
         <v>30000</v>
       </c>
-      <c r="AA71" s="13" t="inlineStr">
-        <is>
-          <t>Readback of the persisted device setting. Requested initial value is 100 Ohm, matching the package default and sustained historian value.</t>
-        </is>
-      </c>
+      <c r="AA71" s="13" t="inlineStr"/>
     </row>
     <row r="72" ht="42" customHeight="1">
       <c r="A72" s="14" t="inlineStr">
@@ -6735,22 +6733,22 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>MeasurementsPerCalculation</t>
+          <t>State</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>Averaging count persisted in package-owned state.</t>
+          <t>Validity state of the installed production calibration tables.</t>
         </is>
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.MeasurementsPerCalculation</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.State</t>
         </is>
       </c>
       <c r="E72" s="14" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F72" s="14" t="inlineStr">
@@ -6768,21 +6766,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I72" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J72" s="14" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="K72" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="L72" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="M72" s="14" t="n">
-        <v>100</v>
-      </c>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="14" t="n"/>
+      <c r="L72" s="14" t="n"/>
+      <c r="M72" s="14" t="n"/>
       <c r="N72" s="14" t="n"/>
       <c r="O72" s="14" t="n"/>
       <c r="P72" s="14" t="n"/>
@@ -6810,11 +6798,7 @@
       <c r="Z72" s="14" t="n">
         <v>30000</v>
       </c>
-      <c r="AA72" s="13" t="inlineStr">
-        <is>
-          <t>OPC UA built-in type UInt32. Requested initial readback matches the packaged default of 100.</t>
-        </is>
-      </c>
+      <c r="AA72" s="13" t="inlineStr"/>
     </row>
     <row r="73" ht="42" customHeight="1">
       <c r="A73" s="15" t="inlineStr">
@@ -6824,27 +6808,27 @@
       </c>
       <c r="B73" s="15" t="inlineStr">
         <is>
-          <t>LastCalibrationTime</t>
+          <t>ConfiguredThresholdOhm</t>
         </is>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>Newest modification time among production calibration tables.</t>
+          <t>Threshold persisted in package-owned state.</t>
         </is>
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.LastCalibrationTime</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.ConfiguredThresholdOhm</t>
         </is>
       </c>
       <c r="E73" s="15" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="F73" s="15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ohm</t>
         </is>
       </c>
       <c r="G73" s="15" t="inlineStr">
@@ -6857,11 +6841,21 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I73" s="15" t="n"/>
-      <c r="J73" s="15" t="n"/>
-      <c r="K73" s="15" t="n"/>
-      <c r="L73" s="15" t="n"/>
-      <c r="M73" s="15" t="n"/>
+      <c r="I73" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="15" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="K73" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="L73" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="M73" s="15" t="n">
+        <v>100</v>
+      </c>
       <c r="N73" s="15" t="n"/>
       <c r="O73" s="15" t="n"/>
       <c r="P73" s="15" t="n"/>
@@ -6889,32 +6883,36 @@
       <c r="Z73" s="15" t="n">
         <v>30000</v>
       </c>
-      <c r="AA73" s="15" t="inlineStr"/>
+      <c r="AA73" s="15" t="inlineStr">
+        <is>
+          <t>Readback of the persisted device setting. Requested initial value is 100 Ohm, matching the package default and sustained historian value.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="42" customHeight="1">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>Calibration</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>LastCommandResult</t>
+          <t>MeasurementsPerCalculation</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>Result of the most recent canonical write or method call.</t>
+          <t>Averaging count persisted in package-owned state.</t>
         </is>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Configuration.LastCommandResult</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.MeasurementsPerCalculation</t>
         </is>
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="F74" s="14" t="inlineStr">
@@ -6932,11 +6930,21 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I74" s="14" t="n"/>
-      <c r="J74" s="14" t="n"/>
-      <c r="K74" s="14" t="n"/>
-      <c r="L74" s="14" t="n"/>
-      <c r="M74" s="14" t="n"/>
+      <c r="I74" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J74" s="14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="K74" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="L74" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="M74" s="14" t="n">
+        <v>100</v>
+      </c>
       <c r="N74" s="14" t="n"/>
       <c r="O74" s="14" t="n"/>
       <c r="P74" s="14" t="n"/>
@@ -6962,34 +6970,38 @@
         </is>
       </c>
       <c r="Z74" s="14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AA74" s="13" t="inlineStr"/>
+        <v>30000</v>
+      </c>
+      <c r="AA74" s="13" t="inlineStr">
+        <is>
+          <t>OPC UA built-in type UInt32. Requested initial readback matches the packaged default of 100.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="42" customHeight="1">
       <c r="A75" s="14" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Calibration</t>
         </is>
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>LastCalibrationTime</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
         <is>
-          <t>Aggregate endpoint health: OK, Degraded, Failed, or Starting.</t>
+          <t>Newest modification time among production calibration tables.</t>
         </is>
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Overall</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.LastCalibrationTime</t>
         </is>
       </c>
       <c r="E75" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="F75" s="14" t="inlineStr">
@@ -7037,34 +7049,34 @@
         </is>
       </c>
       <c r="Z75" s="14" t="n">
-        <v>1000</v>
+        <v>30000</v>
       </c>
       <c r="AA75" s="13" t="inlineStr"/>
     </row>
     <row r="76" ht="42" customHeight="1">
       <c r="A76" s="14" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Configuration</t>
         </is>
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>LastUpdate</t>
+          <t>LastCommandResult</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>Time aggregate health was last evaluated.</t>
+          <t>Result of the most recent canonical write or method call.</t>
         </is>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.LastUpdate</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Configuration.LastCommandResult</t>
         </is>
       </c>
       <c r="E76" s="14" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F76" s="14" t="inlineStr">
@@ -7106,8 +7118,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y76" s="14" t="n">
-        <v>1000</v>
+      <c r="Y76" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
       </c>
       <c r="Z76" s="14" t="n">
         <v>1000</v>
@@ -7122,17 +7136,17 @@
       </c>
       <c r="B77" s="15" t="inlineStr">
         <is>
-          <t>Measurement</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Aggregate quality of the measurement subtree.</t>
+          <t>Aggregate endpoint health: OK, Degraded, Failed, or Starting.</t>
         </is>
       </c>
       <c r="D77" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Measurement</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Overall</t>
         </is>
       </c>
       <c r="E77" s="15" t="inlineStr">
@@ -7197,22 +7211,22 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Thermal</t>
+          <t>LastUpdate</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of the thermal subtree.</t>
+          <t>Time aggregate health was last evaluated.</t>
         </is>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Thermal</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.LastUpdate</t>
         </is>
       </c>
       <c r="E78" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="F78" s="14" t="inlineStr">
@@ -7254,10 +7268,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y78" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
+      <c r="Y78" s="14" t="n">
+        <v>1000</v>
       </c>
       <c r="Z78" s="14" t="n">
         <v>1000</v>
@@ -7272,17 +7284,17 @@
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Measurement</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of timekeeping.</t>
+          <t>Aggregate quality of the measurement subtree.</t>
         </is>
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Time</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Measurement</t>
         </is>
       </c>
       <c r="E79" s="14" t="inlineStr">
@@ -7347,17 +7359,17 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>OperatingSystem</t>
+          <t>Thermal</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of operating-system telemetry.</t>
+          <t>Aggregate quality of the thermal subtree.</t>
         </is>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.OperatingSystem</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Thermal</t>
         </is>
       </c>
       <c r="E80" s="14" t="inlineStr">
@@ -7410,7 +7422,7 @@
         </is>
       </c>
       <c r="Z80" s="14" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="AA80" s="13" t="inlineStr"/>
     </row>
@@ -7422,17 +7434,17 @@
       </c>
       <c r="B81" s="15" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>Aggregate quality of network monitoring.</t>
+          <t>Aggregate quality of timekeeping.</t>
         </is>
       </c>
       <c r="D81" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Network</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Time</t>
         </is>
       </c>
       <c r="E81" s="15" t="inlineStr">
@@ -7485,7 +7497,7 @@
         </is>
       </c>
       <c r="Z81" s="15" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="AA81" s="15" t="inlineStr"/>
     </row>
@@ -7497,17 +7509,17 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>OperatingSystem</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of storage monitoring.</t>
+          <t>Aggregate quality of operating-system telemetry.</t>
         </is>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Storage</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.OperatingSystem</t>
         </is>
       </c>
       <c r="E82" s="14" t="inlineStr">
@@ -7560,7 +7572,7 @@
         </is>
       </c>
       <c r="Z82" s="14" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="AA82" s="13" t="inlineStr"/>
     </row>
@@ -7572,17 +7584,17 @@
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of runtime and programmable-logic state.</t>
+          <t>Aggregate quality of network monitoring.</t>
         </is>
       </c>
       <c r="D83" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Firmware</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Network</t>
         </is>
       </c>
       <c r="E83" s="14" t="inlineStr">
@@ -7635,7 +7647,7 @@
         </is>
       </c>
       <c r="Z83" s="14" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="AA83" s="13" t="inlineStr"/>
     </row>
@@ -7647,17 +7659,17 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>Services</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of owned services or OPC UA producer processes.</t>
+          <t>Aggregate quality of storage monitoring.</t>
         </is>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Services</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Storage</t>
         </is>
       </c>
       <c r="E84" s="14" t="inlineStr">
@@ -7710,7 +7722,7 @@
         </is>
       </c>
       <c r="Z84" s="14" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="AA84" s="13" t="inlineStr"/>
     </row>
@@ -7722,17 +7734,17 @@
       </c>
       <c r="B85" s="15" t="inlineStr">
         <is>
-          <t>Calibration</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>Aggregate quality of calibration metadata.</t>
+          <t>Aggregate quality of runtime and programmable-logic state.</t>
         </is>
       </c>
       <c r="D85" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Calibration</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Firmware</t>
         </is>
       </c>
       <c r="E85" s="15" t="inlineStr">
@@ -7797,17 +7809,17 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>SDR</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of SDR acquisition.</t>
+          <t>Aggregate quality of owned services or adapter processes.</t>
         </is>
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.SDR</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Services</t>
         </is>
       </c>
       <c r="E86" s="14" t="inlineStr">
@@ -7860,67 +7872,159 @@
         </is>
       </c>
       <c r="Z86" s="14" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AA86" s="13" t="inlineStr"/>
+    </row>
+    <row r="87" ht="42" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>Aggregate quality of calibration metadata.</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Calibration</t>
+        </is>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F87" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G87" s="14" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H87" s="14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I87" s="14" t="n"/>
+      <c r="J87" s="14" t="n"/>
+      <c r="K87" s="14" t="n"/>
+      <c r="L87" s="14" t="n"/>
+      <c r="M87" s="14" t="n"/>
+      <c r="N87" s="14" t="n"/>
+      <c r="O87" s="14" t="n"/>
+      <c r="P87" s="14" t="n"/>
+      <c r="Q87" s="14" t="n"/>
+      <c r="R87" s="14" t="n"/>
+      <c r="S87" s="14" t="n"/>
+      <c r="T87" s="14" t="n"/>
+      <c r="U87" s="14" t="n"/>
+      <c r="V87" s="14" t="n"/>
+      <c r="W87" s="14" t="inlineStr">
+        <is>
+          <t>Read-Only</t>
+        </is>
+      </c>
+      <c r="X87" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y87" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
+      </c>
+      <c r="Z87" s="14" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AA87" s="13" t="inlineStr"/>
+    </row>
+    <row r="88" ht="42" customHeight="1">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>SDR</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Aggregate quality of SDR acquisition.</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.SDR</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F88" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G88" s="14" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H88" s="14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I88" s="14" t="n"/>
+      <c r="J88" s="14" t="n"/>
+      <c r="K88" s="14" t="n"/>
+      <c r="L88" s="14" t="n"/>
+      <c r="M88" s="14" t="n"/>
+      <c r="N88" s="14" t="n"/>
+      <c r="O88" s="14" t="n"/>
+      <c r="P88" s="14" t="n"/>
+      <c r="Q88" s="14" t="n"/>
+      <c r="R88" s="14" t="n"/>
+      <c r="S88" s="14" t="n"/>
+      <c r="T88" s="14" t="n"/>
+      <c r="U88" s="14" t="n"/>
+      <c r="V88" s="14" t="n"/>
+      <c r="W88" s="14" t="inlineStr">
+        <is>
+          <t>Read-Only</t>
+        </is>
+      </c>
+      <c r="X88" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y88" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
+      </c>
+      <c r="Z88" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="AA86" s="13" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="11" t="n"/>
-      <c r="B87" s="11" t="n"/>
-      <c r="C87" s="11" t="n"/>
-      <c r="D87" s="11" t="n"/>
-      <c r="E87" s="11" t="n"/>
-      <c r="F87" s="11" t="n"/>
-      <c r="G87" s="11" t="n"/>
-      <c r="H87" s="11" t="n"/>
-      <c r="I87" s="11" t="n"/>
-      <c r="J87" s="11" t="n"/>
-      <c r="K87" s="11" t="n"/>
-      <c r="L87" s="11" t="n"/>
-      <c r="M87" s="11" t="n"/>
-      <c r="N87" s="11" t="n"/>
-      <c r="O87" s="11" t="n"/>
-      <c r="P87" s="11" t="n"/>
-      <c r="Q87" s="11" t="n"/>
-      <c r="R87" s="11" t="n"/>
-      <c r="S87" s="11" t="n"/>
-      <c r="T87" s="11" t="n"/>
-      <c r="U87" s="11" t="n"/>
-      <c r="V87" s="11" t="n"/>
-      <c r="W87" s="11" t="n"/>
-      <c r="X87" s="11" t="n"/>
-      <c r="Y87" s="11" t="n"/>
-      <c r="Z87" s="11" t="n"/>
-      <c r="AA87" s="11" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="11" t="n"/>
-      <c r="B88" s="11" t="n"/>
-      <c r="C88" s="11" t="n"/>
-      <c r="D88" s="11" t="n"/>
-      <c r="E88" s="11" t="n"/>
-      <c r="F88" s="11" t="n"/>
-      <c r="G88" s="11" t="n"/>
-      <c r="H88" s="11" t="n"/>
-      <c r="I88" s="11" t="n"/>
-      <c r="J88" s="11" t="n"/>
-      <c r="K88" s="11" t="n"/>
-      <c r="L88" s="11" t="n"/>
-      <c r="M88" s="11" t="n"/>
-      <c r="N88" s="11" t="n"/>
-      <c r="O88" s="11" t="n"/>
-      <c r="P88" s="11" t="n"/>
-      <c r="Q88" s="11" t="n"/>
-      <c r="R88" s="11" t="n"/>
-      <c r="S88" s="11" t="n"/>
-      <c r="T88" s="11" t="n"/>
-      <c r="U88" s="11" t="n"/>
-      <c r="V88" s="11" t="n"/>
-      <c r="W88" s="11" t="n"/>
-      <c r="X88" s="11" t="n"/>
-      <c r="Y88" s="11" t="n"/>
-      <c r="Z88" s="11" t="n"/>
-      <c r="AA88" s="11" t="n"/>
+      <c r="AA88" s="13" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="11" t="n"/>
@@ -11287,7 +11391,7 @@
       <c r="AA204" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA86"/>
+  <autoFilter ref="A1:AA88"/>
   <dataValidations count="5">
     <dataValidation sqref="E2:E204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." type="list">
       <formula1>"Boolean,Byte,Short,Integer,Long,Float,Double,String,DateTime"</formula1>
@@ -11309,7 +11413,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;BGIZMo Kria — K26 SOM / KR260 implementation</oddHeader>
-    <oddFooter>&amp;LDraft 0.7 — GIZMo OPC UA-to-Ignition requirements&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDraft 0.9 — GIZMo OPC UA-to-Ignition requirements&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Define hardware-neutral GIZMo OPC UA contract
</commit_message>
<xml_diff>
--- a/deliverables/GIZMo_Kria_DCS_Intake.xlsx
+++ b/deliverables/GIZMo_Kria_DCS_Intake.xlsx
@@ -10,9 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag List" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tag List'!$A$1:$AA$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tag List'!$A$1:$AA$88</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Tag List'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Tag List'!$A$1:$AA$86</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Tag List'!$A$1:$AA$88</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -614,7 +614,7 @@
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
-          <t>opc.tcp://&lt;assigned-host&gt;:4840 (final host/IP assigned by Slow Controls)</t>
+          <t>opc.tcp://&lt;assigned-host&gt;:4840 (final production host/IP assigned by Slow Controls)</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>Stable string NodeIds; resolve namespace URI at connection time; do not hard-code namespace index.</t>
+          <t>This ICD defines the authoritative, hardware-neutral urn:fnal:gizmo contract. Any GIZMo hardware implementation must conform to its stable string NodeIds, node classes, datatypes, ranks, units, meanings, quality/timestamp rules, and method signatures. Resolve the namespace URI at connection time; do not hard-code its namespace index.</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>Control rows are listed first and color-coded. Green Read-Write rows are bounded configuration setpoints; amber Write-Only rows are typed OPC UA Methods. Read-Only measurement/status rows are device readbacks and must not be writable. Notes identify implemented versus commissioning-gated capabilities.</t>
+          <t>DCS Access records the effective Kria integration profile. Read-Write rows are bounded configuration variables; Write-Only rows are typed OPC UA Methods; Read-Only rows are device readbacks. Contract shape and runtime authorization are separate: Notes distinguish current model 1.3.1 behavior, future model proposals, and commissioning gates.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>Draft 0.8 requirements intake for joint GIZMo / Slow Controls review</t>
+          <t>Draft 0.10 requirements intake for joint GIZMo / Slow Controls review</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Kria values use the retained 2026-07-27..2026-08-03 permanent SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from the connected ZedBoard on 2026-08-12 plus 27 contiguous validation-adapter cycles on 2026-08-13; target communication was lost before the 100-cycle acceptance run completed. These sources refine nominal/desired fields but do not replace approved alarm or metrology limits.</t>
+          <t>Kria values use the retained 2026-07-27..2026-08-03 SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from 2026-08-12 and 27 contiguous off-board adapter-pilot cycles from 2026-08-13. No target-native ZedBoard OPC UA deployment or authenticated write is accepted as evidence in this revision. These sources refine nominal/desired fields but do not replace approved alarm or metrology limits.</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Engineering units ONLY (degC, V, A, psia, bar...). Do NOT put units in the value columns.</t>
+          <t>EngineeringUnits value from the OPC UA contract (for example Cel, V, A, psia, bar). Do not put units in numeric value columns.</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="19" t="n">
-        <v>1000000</v>
+        <v>1023</v>
       </c>
       <c r="K2" s="19" t="n">
         <v>100</v>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="AA2" s="21" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. OPC UA UInt32 accepts 0..1,000,000 Ohm. The requested initial/normal setpoint is 100 Ohm, matching the package default and sustained historian value; the initial authorized operator range is 1..500 Ohm. Zero is accepted by firmware but excluded from the operator range because it effectively disables the resistance-threshold branch. Enforce site authorization and verify Measurement.ThresholdOhm after the write.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. OPC UA UInt32 accepts 0..1023 Ohm. The requested initial/normal setpoint is 100 Ohm, matching the package default and sustained historian value; the initial authorized operator range is 1..500 Ohm. Zero is accepted by firmware but excluded from the operator range because it effectively disables the resistance-threshold branch. Enforce site authorization and verify Measurement.ThresholdOhm after the write.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="AA3" s="21" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. OPC UA UInt32 and ZMon accept 1..1,000,000 reads; requested initial/normal value and packaged default are 100. Normal-operator write; verify Measurement.AveragesPerCalculation and a fresh Sequence afterwards.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. OPC UA UInt32 and ZMon accept 1..1,000,000 reads; requested initial/normal value and packaged default are 100. Normal-operator write; verify Measurement.AveragesPerCalculation and a fresh Sequence afterwards.</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       <c r="Z4" s="23" t="n"/>
       <c r="AA4" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. OPC UA Method: no input; String result. Normal-operator command; clearing a latch shall not suppress an active physical alarm. Audit through the required model-1.4 command-status nodes.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. OPC UA Method: no input; String result. Normal-operator command; clearing a latch shall not suppress an active physical alarm. Audit through the required model-1.4 command-status nodes.</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="F5" s="26" t="inlineStr">
@@ -1567,7 +1567,7 @@
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="26" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: UInt32 reads_per_point input in 1..1,000,000; String acceptance result. Enable for SC only after exclusive hardware ownership, progress/result readback, abort, safe restoration, and controlled calibration activation are commissioned. Never automatic.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: UInt32 reads_per_point input in 1..1,000,000; String acceptance result. Enable for SC only after exclusive hardware ownership, progress/result readback, abort, safe restoration, and controlled calibration activation are commissioned. Never automatic.</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       <c r="Z6" s="23" t="n"/>
       <c r="AA6" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: no input; String result. Output size, timeout, ownership, and return to normal acquisition shall be bounded and audited.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: no input; String result. Output size, timeout, ownership, and return to normal acquisition shall be bounded and audited.</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       <c r="Z7" s="23" t="n"/>
       <c r="AA7" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: no input; String result. This is not a traceable calibration and shall not be presented as one.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: no input; String result. This is not a traceable calibration and shall not be presented as one.</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       <c r="Z8" s="23" t="n"/>
       <c r="AA8" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: absolute DateTime input; String result. Allowed only when the approved time source cannot recover; verify Time.CurrentUtc/Quality afterwards. Does not assert NTP synchronization.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: absolute DateTime input; String result. Allowed only when the approved time source cannot recover; verify Time.CurrentUtc/Quality afterwards. Does not assert NTP synchronization.</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Organization responsible for the GIZMo runtime package and canonical information model.</t>
+          <t>Organization responsible for this GIZMo implementation.</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="AA26" s="13" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. Published value: Fermi National Accelerator Laboratory.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. Published value: Fermi National Accelerator Laboratory.</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>Canonical OPC UA namespace URI.</t>
+          <t>Namespace URI of the hardware-neutral GIZMo–SC OPC UA contract defined by the ICD.</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Semantic version of the canonical OPC UA information model.</t>
+          <t>Semantic version of the hardware-neutral GIZMo–SC OPC UA contract implemented by this producer.</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Installed GIZMo runtime or OPC UA producer version.</t>
+          <t>Installed version of this hardware implementation's GIZMo runtime.</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Boot identifier; changes after target or OPC UA producer restart as defined by the platform.</t>
+          <t>Boot identifier for this hardware instance; changes after its controller boots.</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>Publication date of the canonical OPC UA information model.</t>
+          <t>Publication date of the hardware-neutral GIZMo–SC OPC UA contract version.</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="AA34" s="13" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. The published model date is 2026-07-27 UTC.</t>
+          <t>CONTRACT MODEL 1.3.1. Published 2026-08-13 UTC.</t>
         </is>
       </c>
     </row>
@@ -4348,7 +4348,7 @@
         <v>0</v>
       </c>
       <c r="J42" s="14" t="n">
-        <v>1000000</v>
+        <v>1023</v>
       </c>
       <c r="K42" s="14" t="n">
         <v>100</v>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="F59" s="14" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>Cel</t>
         </is>
       </c>
       <c r="G59" s="14" t="inlineStr">
@@ -5801,7 +5801,7 @@
       </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>Cel</t>
         </is>
       </c>
       <c r="G60" s="14" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="F61" s="15" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>Cel</t>
         </is>
       </c>
       <c r="G61" s="15" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="F62" s="14" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>Cel</t>
         </is>
       </c>
       <c r="G62" s="14" t="inlineStr">
@@ -6095,7 +6095,11 @@
       <c r="Z63" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="AA63" s="13" t="inlineStr"/>
+      <c r="AA63" s="13" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED. The Kria systemd-timesyncd client queries the directly connected Fermilab-synchronized controls workstation. Manual SetSystemTime is a maintenance fallback, not normal operation.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="42" customHeight="1">
       <c r="A64" s="14" t="inlineStr">
@@ -6105,27 +6109,27 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>UptimeSeconds</t>
+          <t>NtpServiceActive</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>Linux uptime.</t>
+          <t>True when the platform network-time client is running.</t>
         </is>
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.UptimeSeconds</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.NtpServiceActive</t>
         </is>
       </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G64" s="14" t="inlineStr">
@@ -6162,43 +6166,49 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y64" s="14" t="n">
-        <v>10000</v>
+      <c r="Y64" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
       </c>
       <c r="Z64" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="AA64" s="13" t="inlineStr"/>
+      <c r="AA64" s="13" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED. Use with NtpSynchronized and Time.Quality; an active client does not by itself prove valid time.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="42" customHeight="1">
       <c r="A65" s="15" t="inlineStr">
         <is>
-          <t>OperatingSystem</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>CpuUtilizationPercent</t>
+          <t>NtpService</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>CPU utilization between samples.</t>
+          <t>Bounded identification of the configured time synchronization service/source.</t>
         </is>
       </c>
       <c r="D65" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.CpuUtilizationPercent</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.NtpService</t>
         </is>
       </c>
       <c r="E65" s="15" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
@@ -6211,21 +6221,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I65" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="K65" s="15" t="n">
-        <v>35.7</v>
-      </c>
-      <c r="L65" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="M65" s="15" t="n">
-        <v>45</v>
-      </c>
+      <c r="I65" s="15" t="n"/>
+      <c r="J65" s="15" t="n"/>
+      <c r="K65" s="15" t="n"/>
+      <c r="L65" s="15" t="n"/>
+      <c r="M65" s="15" t="n"/>
       <c r="N65" s="15" t="n"/>
       <c r="O65" s="15" t="n"/>
       <c r="P65" s="15" t="n"/>
@@ -6245,47 +6245,49 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y65" s="15" t="n">
-        <v>10000</v>
+      <c r="Y65" s="15" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
       </c>
       <c r="Z65" s="15" t="n">
         <v>10000</v>
       </c>
       <c r="AA65" s="15" t="inlineStr">
         <is>
-          <t>Provisional steady-state commissioning envelope from the retained Kria historian: median 35.68%, 1st--99th percentile minute means 34.30--36.66%; short startup/intervention excursions reached 85.47%. Trend only; no utilization alarm is requested.</t>
+          <t>IMPLEMENTED diagnostic readback. No credentials or unrestricted daemon output are exposed.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="42" customHeight="1">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>OperatingSystem</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>MemoryAvailableBytes</t>
+          <t>UptimeSeconds</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>Physical memory available without swapping.</t>
+          <t>Linux uptime.</t>
         </is>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.MemoryAvailableBytes</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Time.UptimeSeconds</t>
         </is>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
-          <t>byte</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G66" s="14" t="inlineStr">
@@ -6298,19 +6300,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I66" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="I66" s="14" t="n"/>
       <c r="J66" s="14" t="n"/>
-      <c r="K66" s="14" t="n">
-        <v>3170000000</v>
-      </c>
-      <c r="L66" s="14" t="n">
-        <v>2500000000</v>
-      </c>
-      <c r="M66" s="14" t="n">
-        <v>3400000000</v>
-      </c>
+      <c r="K66" s="14" t="n"/>
+      <c r="L66" s="14" t="n"/>
+      <c r="M66" s="14" t="n"/>
       <c r="N66" s="14" t="n"/>
       <c r="O66" s="14" t="n"/>
       <c r="P66" s="14" t="n"/>
@@ -6334,43 +6328,39 @@
         <v>10000</v>
       </c>
       <c r="Z66" s="14" t="n">
-        <v>10000</v>
-      </c>
-      <c r="AA66" s="13" t="inlineStr">
-        <is>
-          <t>OPC UA built-in type UInt64. Provisional commissioning envelope from the retained Kria historian: median 3.171e9 bytes; absolute observed 2.522e9--3.362e9 bytes. Trend only; no memory alarm is requested.</t>
-        </is>
-      </c>
+        <v>1000</v>
+      </c>
+      <c r="AA66" s="13" t="inlineStr"/>
     </row>
     <row r="67" ht="42" customHeight="1">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>OperatingSystem</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>RuntimeVersion</t>
+          <t>CpuUtilizationPercent</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
         <is>
-          <t>Installed gizmo-runtime package version.</t>
+          <t>CPU utilization between samples.</t>
         </is>
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.RuntimeVersion</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.CpuUtilizationPercent</t>
         </is>
       </c>
       <c r="E67" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="F67" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>%</t>
         </is>
       </c>
       <c r="G67" s="14" t="inlineStr">
@@ -6383,11 +6373,21 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I67" s="14" t="n"/>
-      <c r="J67" s="14" t="n"/>
-      <c r="K67" s="14" t="n"/>
-      <c r="L67" s="14" t="n"/>
-      <c r="M67" s="14" t="n"/>
+      <c r="I67" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="K67" s="14" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="L67" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="M67" s="14" t="n">
+        <v>45</v>
+      </c>
       <c r="N67" s="14" t="n"/>
       <c r="O67" s="14" t="n"/>
       <c r="P67" s="14" t="n"/>
@@ -6407,45 +6407,47 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y67" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
+      <c r="Y67" s="14" t="n">
+        <v>10000</v>
       </c>
       <c r="Z67" s="14" t="n">
-        <v>30000</v>
-      </c>
-      <c r="AA67" s="13" t="inlineStr"/>
+        <v>10000</v>
+      </c>
+      <c r="AA67" s="13" t="inlineStr">
+        <is>
+          <t>Provisional steady-state commissioning envelope from the retained Kria historian: median 35.68%, 1st--99th percentile minute means 34.30--36.66%; short startup/intervention excursions reached 85.47%. Trend only; no utilization alarm is requested.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="42" customHeight="1">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>OperatingSystem</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>OverlayState</t>
+          <t>MemoryAvailableBytes</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
         <is>
-          <t>FPGA overlay state: Running, Degraded, Missing, or unconfirmed.</t>
+          <t>Physical memory available without swapping.</t>
         </is>
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayState</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.OperatingSystem.MemoryAvailableBytes</t>
         </is>
       </c>
       <c r="E68" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>byte</t>
         </is>
       </c>
       <c r="G68" s="14" t="inlineStr">
@@ -6458,11 +6460,19 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I68" s="14" t="n"/>
+      <c r="I68" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="J68" s="14" t="n"/>
-      <c r="K68" s="14" t="n"/>
-      <c r="L68" s="14" t="n"/>
-      <c r="M68" s="14" t="n"/>
+      <c r="K68" s="14" t="n">
+        <v>3170000000</v>
+      </c>
+      <c r="L68" s="14" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="M68" s="14" t="n">
+        <v>3400000000</v>
+      </c>
       <c r="N68" s="14" t="n"/>
       <c r="O68" s="14" t="n"/>
       <c r="P68" s="14" t="n"/>
@@ -6482,15 +6492,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y68" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
+      <c r="Y68" s="14" t="n">
+        <v>10000</v>
       </c>
       <c r="Z68" s="14" t="n">
-        <v>30000</v>
-      </c>
-      <c r="AA68" s="13" t="inlineStr"/>
+        <v>10000</v>
+      </c>
+      <c r="AA68" s="13" t="inlineStr">
+        <is>
+          <t>OPC UA built-in type UInt64. Provisional commissioning envelope from the retained Kria historian: median 3.171e9 bytes; absolute observed 2.522e9--3.362e9 bytes. Trend only; no memory alarm is requested.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="42" customHeight="1">
       <c r="A69" s="15" t="inlineStr">
@@ -6500,17 +6512,17 @@
       </c>
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>OverlayBitstreamSha256</t>
+          <t>RuntimeVersion</t>
         </is>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>SHA-256 digest of the installed FPGA bitstream.</t>
+          <t>Installed gizmo-runtime package version.</t>
         </is>
       </c>
       <c r="D69" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayBitstreamSha256</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.RuntimeVersion</t>
         </is>
       </c>
       <c r="E69" s="15" t="inlineStr">
@@ -6554,10 +6566,14 @@
       </c>
       <c r="X69" s="15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Y69" s="15" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y69" s="15" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
+      </c>
       <c r="Z69" s="15" t="n">
         <v>30000</v>
       </c>
@@ -6566,22 +6582,22 @@
     <row r="70" ht="42" customHeight="1">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>Calibration</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>OverlayState</t>
         </is>
       </c>
       <c r="C70" s="14" t="inlineStr">
         <is>
-          <t>Validity state of the installed production calibration tables.</t>
+          <t>FPGA overlay state: Running, Degraded, Missing, or unconfirmed.</t>
         </is>
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.State</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayState</t>
         </is>
       </c>
       <c r="E70" s="14" t="inlineStr">
@@ -6641,32 +6657,32 @@
     <row r="71" ht="42" customHeight="1">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>Calibration</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>ConfiguredThresholdOhm</t>
+          <t>OverlayBitstreamSha256</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
-          <t>Threshold persisted in package-owned state.</t>
+          <t>SHA-256 digest of the installed FPGA bitstream.</t>
         </is>
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.ConfiguredThresholdOhm</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Firmware.OverlayBitstreamSha256</t>
         </is>
       </c>
       <c r="E71" s="14" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F71" s="14" t="inlineStr">
         <is>
-          <t>Ohm</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G71" s="14" t="inlineStr">
@@ -6679,21 +6695,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I71" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" s="14" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="K71" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="L71" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="M71" s="14" t="n">
-        <v>100</v>
-      </c>
+      <c r="I71" s="14" t="n"/>
+      <c r="J71" s="14" t="n"/>
+      <c r="K71" s="14" t="n"/>
+      <c r="L71" s="14" t="n"/>
+      <c r="M71" s="14" t="n"/>
       <c r="N71" s="14" t="n"/>
       <c r="O71" s="14" t="n"/>
       <c r="P71" s="14" t="n"/>
@@ -6710,22 +6716,14 @@
       </c>
       <c r="X71" s="14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Y71" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y71" s="14" t="n"/>
       <c r="Z71" s="14" t="n">
         <v>30000</v>
       </c>
-      <c r="AA71" s="13" t="inlineStr">
-        <is>
-          <t>Readback of the persisted device setting. Requested initial value is 100 Ohm, matching the package default and sustained historian value.</t>
-        </is>
-      </c>
+      <c r="AA71" s="13" t="inlineStr"/>
     </row>
     <row r="72" ht="42" customHeight="1">
       <c r="A72" s="14" t="inlineStr">
@@ -6735,22 +6733,22 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>MeasurementsPerCalculation</t>
+          <t>State</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>Averaging count persisted in package-owned state.</t>
+          <t>Validity state of the installed production calibration tables.</t>
         </is>
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.MeasurementsPerCalculation</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.State</t>
         </is>
       </c>
       <c r="E72" s="14" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F72" s="14" t="inlineStr">
@@ -6768,21 +6766,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I72" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J72" s="14" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="K72" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="L72" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="M72" s="14" t="n">
-        <v>100</v>
-      </c>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="14" t="n"/>
+      <c r="L72" s="14" t="n"/>
+      <c r="M72" s="14" t="n"/>
       <c r="N72" s="14" t="n"/>
       <c r="O72" s="14" t="n"/>
       <c r="P72" s="14" t="n"/>
@@ -6810,11 +6798,7 @@
       <c r="Z72" s="14" t="n">
         <v>30000</v>
       </c>
-      <c r="AA72" s="13" t="inlineStr">
-        <is>
-          <t>OPC UA built-in type UInt32. Requested initial readback matches the packaged default of 100.</t>
-        </is>
-      </c>
+      <c r="AA72" s="13" t="inlineStr"/>
     </row>
     <row r="73" ht="42" customHeight="1">
       <c r="A73" s="15" t="inlineStr">
@@ -6824,27 +6808,27 @@
       </c>
       <c r="B73" s="15" t="inlineStr">
         <is>
-          <t>LastCalibrationTime</t>
+          <t>ConfiguredThresholdOhm</t>
         </is>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>Newest modification time among production calibration tables.</t>
+          <t>Threshold persisted in package-owned state.</t>
         </is>
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.LastCalibrationTime</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.ConfiguredThresholdOhm</t>
         </is>
       </c>
       <c r="E73" s="15" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="F73" s="15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ohm</t>
         </is>
       </c>
       <c r="G73" s="15" t="inlineStr">
@@ -6857,11 +6841,21 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I73" s="15" t="n"/>
-      <c r="J73" s="15" t="n"/>
-      <c r="K73" s="15" t="n"/>
-      <c r="L73" s="15" t="n"/>
-      <c r="M73" s="15" t="n"/>
+      <c r="I73" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="15" t="n">
+        <v>1023</v>
+      </c>
+      <c r="K73" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="L73" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="M73" s="15" t="n">
+        <v>100</v>
+      </c>
       <c r="N73" s="15" t="n"/>
       <c r="O73" s="15" t="n"/>
       <c r="P73" s="15" t="n"/>
@@ -6889,32 +6883,36 @@
       <c r="Z73" s="15" t="n">
         <v>30000</v>
       </c>
-      <c r="AA73" s="15" t="inlineStr"/>
+      <c r="AA73" s="15" t="inlineStr">
+        <is>
+          <t>Readback of the persisted device setting. Requested initial value is 100 Ohm, matching the package default and sustained historian value.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="42" customHeight="1">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>Calibration</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>LastCommandResult</t>
+          <t>MeasurementsPerCalculation</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>Result of the most recent canonical write or method call.</t>
+          <t>Averaging count persisted in package-owned state.</t>
         </is>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Configuration.LastCommandResult</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.MeasurementsPerCalculation</t>
         </is>
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="F74" s="14" t="inlineStr">
@@ -6932,11 +6930,21 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I74" s="14" t="n"/>
-      <c r="J74" s="14" t="n"/>
-      <c r="K74" s="14" t="n"/>
-      <c r="L74" s="14" t="n"/>
-      <c r="M74" s="14" t="n"/>
+      <c r="I74" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J74" s="14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="K74" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="L74" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="M74" s="14" t="n">
+        <v>100</v>
+      </c>
       <c r="N74" s="14" t="n"/>
       <c r="O74" s="14" t="n"/>
       <c r="P74" s="14" t="n"/>
@@ -6962,34 +6970,38 @@
         </is>
       </c>
       <c r="Z74" s="14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AA74" s="13" t="inlineStr"/>
+        <v>30000</v>
+      </c>
+      <c r="AA74" s="13" t="inlineStr">
+        <is>
+          <t>OPC UA built-in type UInt32. Requested initial readback matches the packaged default of 100.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="42" customHeight="1">
       <c r="A75" s="14" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Calibration</t>
         </is>
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>LastCalibrationTime</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
         <is>
-          <t>Aggregate endpoint health: OK, Degraded, Failed, or Starting.</t>
+          <t>Newest modification time among production calibration tables.</t>
         </is>
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Overall</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Calibration.LastCalibrationTime</t>
         </is>
       </c>
       <c r="E75" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="F75" s="14" t="inlineStr">
@@ -7037,34 +7049,34 @@
         </is>
       </c>
       <c r="Z75" s="14" t="n">
-        <v>1000</v>
+        <v>30000</v>
       </c>
       <c r="AA75" s="13" t="inlineStr"/>
     </row>
     <row r="76" ht="42" customHeight="1">
       <c r="A76" s="14" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Configuration</t>
         </is>
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>LastUpdate</t>
+          <t>LastCommandResult</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>Time aggregate health was last evaluated.</t>
+          <t>Result of the most recent canonical write or method call.</t>
         </is>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.LastUpdate</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Configuration.LastCommandResult</t>
         </is>
       </c>
       <c r="E76" s="14" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>String</t>
         </is>
       </c>
       <c r="F76" s="14" t="inlineStr">
@@ -7106,8 +7118,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y76" s="14" t="n">
-        <v>1000</v>
+      <c r="Y76" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
       </c>
       <c r="Z76" s="14" t="n">
         <v>1000</v>
@@ -7122,17 +7136,17 @@
       </c>
       <c r="B77" s="15" t="inlineStr">
         <is>
-          <t>Measurement</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Aggregate quality of the measurement subtree.</t>
+          <t>Aggregate endpoint health: OK, Degraded, Failed, or Starting.</t>
         </is>
       </c>
       <c r="D77" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Measurement</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Overall</t>
         </is>
       </c>
       <c r="E77" s="15" t="inlineStr">
@@ -7197,22 +7211,22 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Thermal</t>
+          <t>LastUpdate</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of the thermal subtree.</t>
+          <t>Time aggregate health was last evaluated.</t>
         </is>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Thermal</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.LastUpdate</t>
         </is>
       </c>
       <c r="E78" s="14" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="F78" s="14" t="inlineStr">
@@ -7254,10 +7268,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y78" s="14" t="inlineStr">
-        <is>
-          <t>On-Change</t>
-        </is>
+      <c r="Y78" s="14" t="n">
+        <v>1000</v>
       </c>
       <c r="Z78" s="14" t="n">
         <v>1000</v>
@@ -7272,17 +7284,17 @@
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Measurement</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of timekeeping.</t>
+          <t>Aggregate quality of the measurement subtree.</t>
         </is>
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Time</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Measurement</t>
         </is>
       </c>
       <c r="E79" s="14" t="inlineStr">
@@ -7347,17 +7359,17 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>OperatingSystem</t>
+          <t>Thermal</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of operating-system telemetry.</t>
+          <t>Aggregate quality of the thermal subtree.</t>
         </is>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.OperatingSystem</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Thermal</t>
         </is>
       </c>
       <c r="E80" s="14" t="inlineStr">
@@ -7410,7 +7422,7 @@
         </is>
       </c>
       <c r="Z80" s="14" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="AA80" s="13" t="inlineStr"/>
     </row>
@@ -7422,17 +7434,17 @@
       </c>
       <c r="B81" s="15" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>Aggregate quality of network monitoring.</t>
+          <t>Aggregate quality of timekeeping.</t>
         </is>
       </c>
       <c r="D81" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Network</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Time</t>
         </is>
       </c>
       <c r="E81" s="15" t="inlineStr">
@@ -7485,7 +7497,7 @@
         </is>
       </c>
       <c r="Z81" s="15" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="AA81" s="15" t="inlineStr"/>
     </row>
@@ -7497,17 +7509,17 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>OperatingSystem</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of storage monitoring.</t>
+          <t>Aggregate quality of operating-system telemetry.</t>
         </is>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Storage</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.OperatingSystem</t>
         </is>
       </c>
       <c r="E82" s="14" t="inlineStr">
@@ -7560,7 +7572,7 @@
         </is>
       </c>
       <c r="Z82" s="14" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="AA82" s="13" t="inlineStr"/>
     </row>
@@ -7572,17 +7584,17 @@
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of runtime and programmable-logic state.</t>
+          <t>Aggregate quality of network monitoring.</t>
         </is>
       </c>
       <c r="D83" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Firmware</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Network</t>
         </is>
       </c>
       <c r="E83" s="14" t="inlineStr">
@@ -7635,7 +7647,7 @@
         </is>
       </c>
       <c r="Z83" s="14" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="AA83" s="13" t="inlineStr"/>
     </row>
@@ -7647,17 +7659,17 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>Services</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of owned services or OPC UA producer processes.</t>
+          <t>Aggregate quality of storage monitoring.</t>
         </is>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Services</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Storage</t>
         </is>
       </c>
       <c r="E84" s="14" t="inlineStr">
@@ -7710,7 +7722,7 @@
         </is>
       </c>
       <c r="Z84" s="14" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="AA84" s="13" t="inlineStr"/>
     </row>
@@ -7722,17 +7734,17 @@
       </c>
       <c r="B85" s="15" t="inlineStr">
         <is>
-          <t>Calibration</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>Aggregate quality of calibration metadata.</t>
+          <t>Aggregate quality of runtime and programmable-logic state.</t>
         </is>
       </c>
       <c r="D85" s="15" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Calibration</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Firmware</t>
         </is>
       </c>
       <c r="E85" s="15" t="inlineStr">
@@ -7797,17 +7809,17 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>SDR</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>Aggregate quality of SDR acquisition.</t>
+          <t>Aggregate quality of owned services or adapter processes.</t>
         </is>
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.SDR</t>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Services</t>
         </is>
       </c>
       <c r="E86" s="14" t="inlineStr">
@@ -7860,67 +7872,159 @@
         </is>
       </c>
       <c r="Z86" s="14" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AA86" s="13" t="inlineStr"/>
+    </row>
+    <row r="87" ht="42" customHeight="1">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>Aggregate quality of calibration metadata.</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.Calibration</t>
+        </is>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F87" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G87" s="14" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H87" s="14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I87" s="14" t="n"/>
+      <c r="J87" s="14" t="n"/>
+      <c r="K87" s="14" t="n"/>
+      <c r="L87" s="14" t="n"/>
+      <c r="M87" s="14" t="n"/>
+      <c r="N87" s="14" t="n"/>
+      <c r="O87" s="14" t="n"/>
+      <c r="P87" s="14" t="n"/>
+      <c r="Q87" s="14" t="n"/>
+      <c r="R87" s="14" t="n"/>
+      <c r="S87" s="14" t="n"/>
+      <c r="T87" s="14" t="n"/>
+      <c r="U87" s="14" t="n"/>
+      <c r="V87" s="14" t="n"/>
+      <c r="W87" s="14" t="inlineStr">
+        <is>
+          <t>Read-Only</t>
+        </is>
+      </c>
+      <c r="X87" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y87" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
+      </c>
+      <c r="Z87" s="14" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AA87" s="13" t="inlineStr"/>
+    </row>
+    <row r="88" ht="42" customHeight="1">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>SDR</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Aggregate quality of SDR acquisition.</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>nsu=urn:fnal:gizmo;s=GIZMo.Health.SDR</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="F88" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G88" s="14" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H88" s="14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I88" s="14" t="n"/>
+      <c r="J88" s="14" t="n"/>
+      <c r="K88" s="14" t="n"/>
+      <c r="L88" s="14" t="n"/>
+      <c r="M88" s="14" t="n"/>
+      <c r="N88" s="14" t="n"/>
+      <c r="O88" s="14" t="n"/>
+      <c r="P88" s="14" t="n"/>
+      <c r="Q88" s="14" t="n"/>
+      <c r="R88" s="14" t="n"/>
+      <c r="S88" s="14" t="n"/>
+      <c r="T88" s="14" t="n"/>
+      <c r="U88" s="14" t="n"/>
+      <c r="V88" s="14" t="n"/>
+      <c r="W88" s="14" t="inlineStr">
+        <is>
+          <t>Read-Only</t>
+        </is>
+      </c>
+      <c r="X88" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y88" s="14" t="inlineStr">
+        <is>
+          <t>On-Change</t>
+        </is>
+      </c>
+      <c r="Z88" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="AA86" s="13" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="11" t="n"/>
-      <c r="B87" s="11" t="n"/>
-      <c r="C87" s="11" t="n"/>
-      <c r="D87" s="11" t="n"/>
-      <c r="E87" s="11" t="n"/>
-      <c r="F87" s="11" t="n"/>
-      <c r="G87" s="11" t="n"/>
-      <c r="H87" s="11" t="n"/>
-      <c r="I87" s="11" t="n"/>
-      <c r="J87" s="11" t="n"/>
-      <c r="K87" s="11" t="n"/>
-      <c r="L87" s="11" t="n"/>
-      <c r="M87" s="11" t="n"/>
-      <c r="N87" s="11" t="n"/>
-      <c r="O87" s="11" t="n"/>
-      <c r="P87" s="11" t="n"/>
-      <c r="Q87" s="11" t="n"/>
-      <c r="R87" s="11" t="n"/>
-      <c r="S87" s="11" t="n"/>
-      <c r="T87" s="11" t="n"/>
-      <c r="U87" s="11" t="n"/>
-      <c r="V87" s="11" t="n"/>
-      <c r="W87" s="11" t="n"/>
-      <c r="X87" s="11" t="n"/>
-      <c r="Y87" s="11" t="n"/>
-      <c r="Z87" s="11" t="n"/>
-      <c r="AA87" s="11" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="11" t="n"/>
-      <c r="B88" s="11" t="n"/>
-      <c r="C88" s="11" t="n"/>
-      <c r="D88" s="11" t="n"/>
-      <c r="E88" s="11" t="n"/>
-      <c r="F88" s="11" t="n"/>
-      <c r="G88" s="11" t="n"/>
-      <c r="H88" s="11" t="n"/>
-      <c r="I88" s="11" t="n"/>
-      <c r="J88" s="11" t="n"/>
-      <c r="K88" s="11" t="n"/>
-      <c r="L88" s="11" t="n"/>
-      <c r="M88" s="11" t="n"/>
-      <c r="N88" s="11" t="n"/>
-      <c r="O88" s="11" t="n"/>
-      <c r="P88" s="11" t="n"/>
-      <c r="Q88" s="11" t="n"/>
-      <c r="R88" s="11" t="n"/>
-      <c r="S88" s="11" t="n"/>
-      <c r="T88" s="11" t="n"/>
-      <c r="U88" s="11" t="n"/>
-      <c r="V88" s="11" t="n"/>
-      <c r="W88" s="11" t="n"/>
-      <c r="X88" s="11" t="n"/>
-      <c r="Y88" s="11" t="n"/>
-      <c r="Z88" s="11" t="n"/>
-      <c r="AA88" s="11" t="n"/>
+      <c r="AA88" s="13" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="11" t="n"/>
@@ -11287,7 +11391,7 @@
       <c r="AA204" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA86"/>
+  <autoFilter ref="A1:AA88"/>
   <dataValidations count="5">
     <dataValidation sqref="E2:E204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." type="list">
       <formula1>"Boolean,Byte,Short,Integer,Long,Float,Double,String,DateTime"</formula1>
@@ -11309,7 +11413,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;BGIZMo Kria — K26 SOM / KR260 implementation</oddHeader>
-    <oddFooter>&amp;LDraft 0.7 — GIZMo OPC UA-to-Ignition requirements&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDraft 0.9 — GIZMo OPC UA-to-Ignition requirements&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Define Kria authority and ZedBoard conformance
</commit_message>
<xml_diff>
--- a/deliverables/GIZMo_Kria_DCS_Intake.xlsx
+++ b/deliverables/GIZMo_Kria_DCS_Intake.xlsx
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="B1:C41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>Stable string NodeIds; resolve namespace URI at connection time; do not hard-code namespace index.</t>
+          <t>The generated Kria model 1.3.1 schema is the authoritative GIZMo–Slow Controls contract. Stable string NodeIds, datatypes, units, ranges, access metadata, and meanings are canonical; resolve the namespace URI at connection time and do not hard-code a namespace index. The ZedBoard profile is conforming and non-authoritative.</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>Control rows are listed first and color-coded. Green Read-Write rows are bounded configuration setpoints; amber Write-Only rows are typed OPC UA Methods. Read-Only measurement/status rows are device readbacks and must not be writable. Notes identify implemented versus commissioning-gated capabilities.</t>
+          <t>Control rows are listed first and color-coded. Green Read-Write rows are bounded configuration setpoints; amber Write-Only rows are typed OPC UA Methods. Read-Only measurement/status rows are device readbacks. A narrower ZedBoard accepted subset does not change canonical engineering metadata. Notes identify implemented, development, and commissioning-gated capabilities.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>Draft 0.9 requirements intake for joint GIZMo / Slow Controls review</t>
+          <t>Draft 0.10 requirements intake for joint GIZMo / Slow Controls review</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>DUNE-doc 37315 v.1 bridge/OPC UA/Ignition architecture and June 2026 SC infrastructure/status analysis. Ignition reads each GIZMo OPC UA endpoint directly and owns production tags, alarms, trends, audit, and history; no intermediate history service is requested.</t>
+          <t>DUNE-doc 37315 v.1 bridge/OPC UA/Ignition architecture and June 2026 SC infrastructure/status analysis. Ignition uses two independent connections, reads each GIZMo endpoint directly, and owns production tags, alarms, trends, audit, and history. Neither producer is a fallback, proxy, lifecycle owner, or control path for the other; no intermediate history service is requested.</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Kria values use the retained 2026-07-27..2026-08-03 permanent SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from 2026-08-12, 27 contiguous adapter-pilot cycles, and the 2026-08-13 native-server authenticated 100-Ohm idempotent write/readback. The full 100-cycle physical-display acceptance remains open. These sources refine nominal/desired fields but do not replace approved alarm or metrology limits.</t>
+          <t>Kria values use the retained 2026-07-27..2026-08-03 permanent SQLite replica as observational evidence. Legacy values use 15 direct coherent frames from 2026-08-12, 27 contiguous adapter-pilot cycles, and a 2026-08-13 target-side development-server 100-Ohm idempotent transaction. The ZedBoard server remains in development; the 100-cycle physical-display and production-security acceptance gates remain open. Evidence refines nominal/desired fields but does not replace approved alarm or metrology limits.</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="AA2" s="21" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. OPC UA UInt32 accepts 0..1,000,000 Ohm. The requested initial/normal setpoint is 100 Ohm, matching the package default and sustained historian value; the initial authorized operator range is 1..500 Ohm. Zero is accepted by firmware but excluded from the operator range because it effectively disables the resistance-threshold branch. Enforce site authorization and verify Measurement.ThresholdOhm after the write.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. OPC UA UInt32 accepts 0..1,000,000 Ohm. The requested initial/normal setpoint is 100 Ohm, matching the package default and sustained historian value; the initial authorized operator range is 1..500 Ohm. Zero is accepted by firmware but excluded from the operator range because it effectively disables the resistance-threshold branch. Enforce site authorization and verify Measurement.ThresholdOhm after the write.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="AA3" s="21" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. OPC UA UInt32 and ZMon accept 1..1,000,000 reads; requested initial/normal value and packaged default are 100. Normal-operator write; verify Measurement.AveragesPerCalculation and a fresh Sequence afterwards.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. OPC UA UInt32 and ZMon accept 1..1,000,000 reads; requested initial/normal value and packaged default are 100. Normal-operator write; verify Measurement.AveragesPerCalculation and a fresh Sequence afterwards.</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       <c r="Z4" s="23" t="n"/>
       <c r="AA4" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. OPC UA Method: no input; String result. Normal-operator command; clearing a latch shall not suppress an active physical alarm. Audit through the required model-1.4 command-status nodes.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. OPC UA Method: no input; String result. Normal-operator command; clearing a latch shall not suppress an active physical alarm. Audit through the required model-1.4 command-status nodes.</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="26" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: UInt32 reads_per_point input in 1..1,000,000; String acceptance result. Enable for SC only after exclusive hardware ownership, progress/result readback, abort, safe restoration, and controlled calibration activation are commissioned. Never automatic.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: UInt32 reads_per_point input in 1..1,000,000; String acceptance result. Enable for SC only after exclusive hardware ownership, progress/result readback, abort, safe restoration, and controlled calibration activation are commissioned. Never automatic.</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       <c r="Z6" s="23" t="n"/>
       <c r="AA6" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: no input; String result. Output size, timeout, ownership, and return to normal acquisition shall be bounded and audited.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: no input; String result. Output size, timeout, ownership, and return to normal acquisition shall be bounded and audited.</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       <c r="Z7" s="23" t="n"/>
       <c r="AA7" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: no input; String result. This is not a traceable calibration and shall not be presented as one.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: no input; String result. This is not a traceable calibration and shall not be presented as one.</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       <c r="Z8" s="23" t="n"/>
       <c r="AA8" s="25" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3, MAINTENANCE-ONLY. OPC UA Method: absolute DateTime input; String result. Allowed only when the approved time source cannot recover; verify Time.CurrentUtc/Quality afterwards. Does not assert NTP synchronization.</t>
+          <t>IMPLEMENTED MODEL 1.3.1, MAINTENANCE-ONLY. OPC UA Method: absolute DateTime input; String result. Allowed only when the approved time source cannot recover; verify Time.CurrentUtc/Quality afterwards. Does not assert NTP synchronization.</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="AA26" s="13" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. Published value: Fermi National Accelerator Laboratory.</t>
+          <t>IMPLEMENTED MODEL 1.3.1. Published value: Fermi National Accelerator Laboratory.</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3306,11 @@
       </c>
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="n"/>
-      <c r="K28" s="14" t="n"/>
+      <c r="K28" s="14" t="inlineStr">
+        <is>
+          <t>urn:fnal:gizmo</t>
+        </is>
+      </c>
       <c r="L28" s="14" t="n"/>
       <c r="M28" s="14" t="n"/>
       <c r="N28" s="14" t="n"/>
@@ -3332,7 +3336,11 @@
       <c r="Z28" s="14" t="n">
         <v>30000</v>
       </c>
-      <c r="AA28" s="13" t="inlineStr"/>
+      <c r="AA28" s="13" t="inlineStr">
+        <is>
+          <t>AUTHORITATIVE CONTRACT. Resolve this namespace URI at connection time; never hard-code the runtime namespace index.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
@@ -3377,7 +3385,11 @@
       </c>
       <c r="I29" s="15" t="n"/>
       <c r="J29" s="15" t="n"/>
-      <c r="K29" s="15" t="n"/>
+      <c r="K29" s="15" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
       <c r="L29" s="15" t="n"/>
       <c r="M29" s="15" t="n"/>
       <c r="N29" s="15" t="n"/>
@@ -3403,7 +3415,11 @@
       <c r="Z29" s="15" t="n">
         <v>30000</v>
       </c>
-      <c r="AA29" s="15" t="inlineStr"/>
+      <c r="AA29" s="15" t="inlineStr">
+        <is>
+          <t>AUTHORITATIVE CONTRACT. The Kria-generated model 1.3.1 schema defines the required baseline for both producers.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
@@ -3736,7 +3752,11 @@
       </c>
       <c r="I34" s="14" t="n"/>
       <c r="J34" s="14" t="n"/>
-      <c r="K34" s="14" t="n"/>
+      <c r="K34" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-14T00:00:00Z</t>
+        </is>
+      </c>
       <c r="L34" s="14" t="n"/>
       <c r="M34" s="14" t="n"/>
       <c r="N34" s="14" t="n"/>
@@ -3764,7 +3784,7 @@
       </c>
       <c r="AA34" s="13" t="inlineStr">
         <is>
-          <t>IMPLEMENTED MODEL 1.3. The published model date is 2026-07-27 UTC.</t>
+          <t>AUTHORITATIVE MODEL 1.3.1 publication date.</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4094,7 @@
       </c>
       <c r="AA38" s="13" t="inlineStr">
         <is>
-          <t>Kria validated presentation range: 0..500 Ohm. For a finite InRange value, the requested normal band begins at the 100-Ohm threshold. Normal open-loop operation is instead ResistanceRange=OutOfRange (HIGH Z) with non-good StatusCode plus NaN/null; it is not a fabricated 500-Ohm measurement. Ignition shall alarm from Alarm.Active rather than independently comparing this value. Existing permanent Kria SQLite replica, 2026-07-27 20:57 UTC through 2026-08-03 19:07 UTC (560,762 fast samples and 56,082 platform samples). The database is commissioning evidence only; Ignition remains the production OPC UA client and historian.</t>
+          <t>Kria validated presentation range: 0..500 Ohm. For a finite InRange value, the requested normal band begins at the 100-Ohm threshold. Normal open-loop operation is instead ResistanceRange=OutOfRange (HIGH Z) with Good StatusCode plus NaN/null; HIGH Z is a valid measured range state, not a quality fault or a fabricated 500-Ohm measurement. Ignition shall alarm from Alarm.Active rather than independently comparing this value. Existing permanent Kria SQLite replica, 2026-07-27 20:57 UTC through 2026-08-03 19:07 UTC (560,762 fast samples and 56,082 platform samples). The database is commissioning evidence only; Ignition remains the production OPC UA client and historian.</t>
         </is>
       </c>
     </row>
@@ -11413,7 +11433,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;BGIZMo Kria — K26 SOM / KR260 implementation</oddHeader>
-    <oddFooter>&amp;LDraft 0.9 — GIZMo OPC UA-to-Ignition requirements&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDraft 0.10 — GIZMo OPC UA-to-Ignition requirements&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>